<commit_message>
chore: add custom-CI test result
</commit_message>
<xml_diff>
--- a/scripts/results/known_growth_phenotypes_w_pred.xlsx
+++ b/scripts/results/known_growth_phenotypes_w_pred.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1425,7 +1425,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Acetate</t>
+          <t>6-Phosphogluconate</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="F35" t="inlineStr"/>
       <c r="G35" t="n">
-        <v>0.385</v>
+        <v>-0.032</v>
       </c>
     </row>
     <row r="36">
@@ -1452,18 +1452,18 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Alanine</t>
+          <t>Acetate</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Unsure</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="n">
-        <v>0.585</v>
+        <v>0.385</v>
       </c>
     </row>
     <row r="37">
@@ -1479,18 +1479,18 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Alginate</t>
+          <t>Alanine</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Unsure</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="n">
-        <v>-0.032</v>
+        <v>0.585</v>
       </c>
     </row>
     <row r="38">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Choline</t>
+          <t>Alginate</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="n">
-        <v>0</v>
+        <v>-0.032</v>
       </c>
     </row>
     <row r="39">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Ectoine</t>
+          <t>Choline</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Fructose</t>
+          <t>Ectoine</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1587,18 +1587,18 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Galactose</t>
+          <t>Fructose</t>
         </is>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="n">
-        <v>0.73</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Galacturonic Acid</t>
+          <t>Galactose</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1625,7 +1625,7 @@
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="n">
-        <v>0.645</v>
+        <v>0.73</v>
       </c>
     </row>
     <row r="43">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Glucose </t>
+          <t>Galacturonic Acid</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="n">
-        <v>0.75</v>
+        <v>0.645</v>
       </c>
     </row>
     <row r="44">
@@ -1668,18 +1668,18 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Glucuronic Acid</t>
+          <t xml:space="preserve">Glucose </t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="n">
-        <v>-0.032</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="45">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Glycolate</t>
+          <t>Glucuronic Acid</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
@@ -1706,7 +1706,7 @@
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="n">
-        <v>0</v>
+        <v>-0.032</v>
       </c>
     </row>
     <row r="46">
@@ -1722,13 +1722,13 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Homarine</t>
+          <t>Glycolate</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Unsure</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -1749,18 +1749,18 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Mannuronic Acid</t>
+          <t>Homarine</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Unsure</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="n">
-        <v>0.645</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -1776,18 +1776,18 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Proline</t>
+          <t>Mannuronic Acid</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Unsure</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="n">
-        <v>0.638</v>
+        <v>0.645</v>
       </c>
     </row>
     <row r="49">
@@ -1803,24 +1803,24 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Sucrose</t>
+          <t>Phosphoenolpyruvate</t>
         </is>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="n">
-        <v>0</v>
+        <v>-0.032</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ProMM</t>
+          <t>Minimal Basal Medium (Moran Lab)</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1830,32 +1830,24 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>3-methyl-2-oxobutanoic acid</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Proline</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>(Halloran, 2026)</t>
-        </is>
-      </c>
+          <t>Unsure</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr"/>
       <c r="G50" t="n">
-        <v>0.491</v>
+        <v>0.638</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ProMM</t>
+          <t>Minimal Basal Medium (Moran Lab)</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1865,24 +1857,16 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>3-methyl-2-oxopentanoic acid</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
+          <t>Sucrose</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>(Halloran, 2026)</t>
-        </is>
-      </c>
+      <c r="F51" t="inlineStr"/>
       <c r="G51" t="n">
         <v>0</v>
       </c>
@@ -1900,7 +1884,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>4-hydroxybenzoic acid</t>
+          <t>3-methyl-2-oxobutanoic acid</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1910,7 +1894,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -1919,7 +1903,7 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>0</v>
+        <v>0.491</v>
       </c>
     </row>
     <row r="53">
@@ -1935,7 +1919,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>4-methyl-2-oxopentanoic acid</t>
+          <t>3-methyl-2-oxopentanoic acid</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1970,7 +1954,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Isoleucine</t>
+          <t>4-hydroxybenzoic acid</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1980,7 +1964,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -1989,7 +1973,7 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>0.537</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
@@ -2005,7 +1989,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Kynurenine</t>
+          <t>4-methyl-2-oxopentanoic acid</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -2040,7 +2024,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Leucine</t>
+          <t>Isoleucine</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -2059,7 +2043,7 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>0.499</v>
+        <v>0.537</v>
       </c>
     </row>
     <row r="57">
@@ -2075,7 +2059,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Thymidine</t>
+          <t>Kynurenine</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2110,7 +2094,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Valine</t>
+          <t>Leucine</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2129,13 +2113,13 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>0.47</v>
+        <v>0.499</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Seawater Medium</t>
+          <t>ProMM</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2145,7 +2129,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Phenol</t>
+          <t>Thymidine</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2155,50 +2139,120 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>(Koch, 2020)</t>
+          <t>(Halloran, 2026)</t>
         </is>
       </c>
       <c r="G59" t="n">
-        <v>0.265</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>ProMM</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>NH3</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Valine</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>(Halloran, 2026)</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>0.47</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>Seawater Medium</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>NH3</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>NH3</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Phenol</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>(Koch, 2020)</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>0.265</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Seawater Medium</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>NH3</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
         <is>
           <t>alpha-Mannan</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
         <is>
           <t>(Koch, 2020)</t>
         </is>
       </c>
-      <c r="G60" t="n">
+      <c r="G62" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>